<commit_message>
feat: ServiceRequest/Procedure 加入長照服務項目 coding slice，更名 CS/VS
- LTCServiceRequest.code.coding 新增 ltcServiceItem slice（binding 至 VS_TW_LTC_ServiceItem）
- LTCProcedureCareActivity.code.coding 新增 ltcServiceItem slice，保留繼承的 sct-procedures
- CodeSystem/ValueSet 從「長照 SDK－服務項目」更名為「臺灣長照服務項目」
- 更新範例使用長照 2.0 服務項目代碼（BB03、BA07）
- 更新 IG 網頁（0 errors, 0 warnings）
</commit_message>
<xml_diff>
--- a/docs/CodeSystem-cs-tw-ltc-service-item.xlsx
+++ b/docs/CodeSystem-cs-tw-ltc-service-item.xlsx
@@ -42,7 +42,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>長照 SDK－服務項目代碼</t>
+    <t>臺灣長照服務項目代碼</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-02T13:32:15+08:00</t>
+    <t>2026-04-03T21:17:06+08:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>對應 r4.* 臺灣長照給付『照顧組合／輔具／無障礙修繕』服務項目代碼（AA..FA 系列），來源：清單.xlsx。</t>
+    <t>臺灣長照 2.0 給付之服務項目代碼（AA..GA 系列），涵蓋照顧組合、專業服務、交通接送、喘息服務等項目，適用於長照服務之申請、核定與使用紀錄。</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>